<commit_message>
añadido algunos analisis electricos
</commit_message>
<xml_diff>
--- a/Hardware/Analisis Eléctrico y Térmico/Analisiselectrico-C.xlsx
+++ b/Hardware/Analisis Eléctrico y Térmico/Analisiselectrico-C.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92074c9dfb58844c/Documentos/UNIVERSIDAD/MASTER/1/TPI/SE/TP1-G1/Hardware/Analisis Eléctrico y Térmico/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_BF010325F10992A21E5D2AAF911A502F96B28E63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1438F95-4E96-4A5B-83B8-A584B48BD07F}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="11_BF010325F10992A21E5D2AAF911A502F96B28E63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24B9D9C8-5466-4B1D-9449-86D2C61CD9F1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="62">
   <si>
     <t>TOTAL</t>
   </si>
@@ -182,12 +182,6 @@
       </rPr>
       <t xml:space="preserve"> = 0.8V to 5.0V </t>
     </r>
-  </si>
-  <si>
-    <t>5.0</t>
-  </si>
-  <si>
-    <t>3.3</t>
   </si>
   <si>
     <t>Does not include current through the pull-up resistor on USBDP In USB suspend mode, the D+ voltage can go up to a maximum of 3.8 V.</t>
@@ -271,9 +265,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">100 000 </t>
-  </si>
-  <si>
     <t>TEL0132 </t>
   </si>
   <si>
@@ -302,9 +293,6 @@
   </si>
   <si>
     <t xml:space="preserve">Per supply pin </t>
-  </si>
-  <si>
-    <t>0.55</t>
   </si>
   <si>
     <r>
@@ -438,9 +426,6 @@
     <t>LAMBDA62-8D</t>
   </si>
   <si>
-    <t>39.6</t>
-  </si>
-  <si>
     <r>
       <t>25°C, V</t>
     </r>
@@ -478,10 +463,6 @@
     <t>MCP1725-ADJ E/SN </t>
   </si>
   <si>
-    <t>IL = 0 mA, VIN =  VIN ≥ 2.3V and 
-VIN ≥ VOUT(MAX) + VDROPOUT(MAX), VOUT = 0.8V to 5.0V</t>
-  </si>
-  <si>
     <t>M20-6102045 </t>
   </si>
   <si>
@@ -501,6 +482,52 @@
   </si>
   <si>
     <t>W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">power </t>
+  </si>
+  <si>
+    <t>P_3,3V</t>
+  </si>
+  <si>
+    <t>P_1,2V</t>
+  </si>
+  <si>
+    <t>mW</t>
+  </si>
+  <si>
+    <t>standby power</t>
+  </si>
+  <si>
+    <t>FRD Quad at 133MHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IL = 0 mA, VIN = Note 1,
+VOUT = 0.8V to 5.0V</t>
+  </si>
+  <si>
+    <t>Supply Current</t>
+  </si>
+  <si>
+    <t>P_2,6V</t>
+  </si>
+  <si>
+    <t>MMBT3904-7-F</t>
+  </si>
+  <si>
+    <t>NDS332P</t>
+  </si>
+  <si>
+    <t>S6BZRSM4ATFLFSN</t>
+  </si>
+  <si>
+    <t>M20-6102045</t>
+  </si>
+  <si>
+    <t>ZHR-6</t>
+  </si>
+  <si>
+    <t>P_5V</t>
   </si>
 </sst>
 </file>
@@ -583,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -616,6 +643,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,6 +661,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -896,7 +930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5703125" customWidth="1"/>
@@ -988,104 +1022,152 @@
         <v>1500</v>
       </c>
       <c r="E4">
-        <v>7500</v>
+        <f>C4*D4*(10^(-6))</f>
+        <v>7.4999999999999997E-3</v>
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D5" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="5" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B5" s="7" t="s">
         <v>19</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>220</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E9" si="0">C5*D5*(10^(-6))</f>
+        <v>1.0999999999999998E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
       </c>
       <c r="D6">
-        <v>220</v>
+        <v>18</v>
       </c>
       <c r="E6">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D7" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="2" t="s">
+        <f t="shared" si="0"/>
+        <v>8.9999999999999992E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="8" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D8">
-        <v>18</v>
-      </c>
+      <c r="C7" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="D7"/>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="1"/>
       <c r="E8">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" s="8" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="2" t="s">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="D9" s="2">
+        <v>100000</v>
+      </c>
+      <c r="E9">
+        <f>C9*D9*(10^(-6))</f>
+        <v>0.32999999999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1">
+        <f>SUMIFS(E$4:E$14,C$4:C$14,"5")</f>
+        <v>8.6899999999999998E-3</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" ref="D16:D17" si="1">SUMIFS(E$4:E$14,C$4:C$14,"3,3")</f>
+        <v>0.32999999999999996</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" t="s">
         <v>21</v>
       </c>
-      <c r="D9"/>
-    </row>
-    <row r="10" spans="1:14" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D10" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11">
-        <v>330000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D14" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D17" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="G18" t="s">
-        <v>23</v>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="1">
+        <f>SUMIFS(E$4:E$14,C$4:C$14,"2,6")</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <f>SUM(D15:D17)</f>
+        <v>0.33868999999999994</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D20" s="1">
+        <f>D19*1000</f>
+        <v>338.68999999999994</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1096,10 +1178,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" customWidth="1"/>
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
     <col min="9" max="9" width="17.28515625" customWidth="1"/>
   </cols>
@@ -1164,76 +1246,105 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <f>21*10^(-6)</f>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E12" si="0">C4*D4</f>
-        <v>0</v>
+        <f>C4*D4</f>
+        <v>6.929999999999999E-5</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>42</v>
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
       </c>
       <c r="C5">
         <v>3.3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <f>21*10^(-6)</f>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="E5">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>C5*D5</f>
+        <v>6.929999999999999E-5</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>43</v>
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6">
+        <v>3.3</v>
+      </c>
+      <c r="D6">
+        <f>21*10^(-6)</f>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>45</v>
+        <f>C6*D6</f>
+        <v>6.929999999999999E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7">
+        <v>3.3</v>
+      </c>
+      <c r="D7">
+        <f>21*10^(-6)</f>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="E7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>C7*D7</f>
+        <v>6.929999999999999E-5</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>46</v>
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <f>21*10^(-6)</f>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ref="E8:E16" si="0">C8*D8</f>
+        <v>2.5199999999999999E-5</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>47</v>
+      <c r="A9" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1245,29 +1356,177 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>48</v>
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10">
+        <v>3.3</v>
+      </c>
+      <c r="D10">
+        <f>17*10^(-3)</f>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>49</v>
+        <v>5.6100000000000004E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11">
+        <v>3.3</v>
+      </c>
+      <c r="D11">
+        <f>220*10^(-6)</f>
+        <v>2.1999999999999998E-4</v>
       </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.2599999999999987E-4</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>50</v>
+      <c r="A12" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
       </c>
       <c r="E12">
         <f t="shared" si="0"/>
         <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14">
+        <v>3.3</v>
+      </c>
+      <c r="D14">
+        <f>15*10^(-3)</f>
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>4.9499999999999995E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15">
+        <v>2.6</v>
+      </c>
+      <c r="D15">
+        <f>20*10^(-3)</f>
+        <v>0.02</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>5.2000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"3,3")</f>
+        <v>0.1066032</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"1,2")</f>
+        <v>2.5199999999999999E-5</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"2,6")</f>
+        <v>5.2000000000000005E-2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="1">
+        <f>SUM(C19:C21)</f>
+        <v>0.1586284</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C24" s="1">
+        <f>C23*1000</f>
+        <v>158.6284</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1278,7 +1537,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1323,7 +1582,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>5</v>
@@ -1350,94 +1609,243 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4" s="10"/>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
+      <c r="C4" s="2">
+        <v>3.3</v>
       </c>
       <c r="D4">
         <v>100</v>
       </c>
       <c r="E4">
-        <v>330</v>
+        <f>(C4*D4)/1000</f>
+        <v>0.33</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B5" s="9"/>
-      <c r="C5" s="2" t="s">
-        <v>21</v>
+      <c r="C5" s="2">
+        <v>3.3</v>
       </c>
       <c r="D5">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>39</v>
+      <c r="E5">
+        <f t="shared" ref="E5:E15" si="0">(C5*D5)/1000</f>
+        <v>3.9599999999999996E-2</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>35</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3.3</v>
       </c>
       <c r="D6">
         <v>240</v>
       </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.79200000000000004</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2"/>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
       </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
-        <v>36</v>
+      <c r="D9" s="2">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>21</v>
+        <v>29</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="2"/>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>56</v>
+      </c>
       <c r="C12" s="2"/>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
+      <c r="A14" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"3,3")</f>
+        <v>1.1616</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"5,0")</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="1">
+        <f>SUMIFS(E$4:E$16,C$4:C$16,"2,6")</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1">
+        <f>SUM(D18:D20)</f>
+        <v>1.1616</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D23" s="1">
+        <f>D22*1000</f>
+        <v>1161.5999999999999</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1519,10 +1927,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C4">
         <v>3.3</v>
@@ -1536,23 +1944,41 @@
         <v>2.3099999999999998E-4</v>
       </c>
     </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1">
+        <f>E4</f>
+        <v>2.3099999999999998E-4</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <f>SUM(E4:E5)</f>
         <v>2.3099999999999998E-4</v>
       </c>
-      <c r="F7" t="s">
-        <v>52</v>
+      <c r="F7" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16">
+        <f>E7*1000</f>
+        <v>0.23099999999999998</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>

</xml_diff>